<commit_message>
test: add login test without email and organize test classes
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/apiTestData.xlsx
+++ b/src/test/resources/testData/apiTestData.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="10">
   <si>
     <t>CT</t>
   </si>
@@ -38,6 +38,9 @@
   </si>
   <si>
     <t>asdf1234</t>
+  </si>
+  <si>
+    <t>CT008</t>
   </si>
 </sst>
 </file>
@@ -95,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -113,6 +116,12 @@
     </xf>
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -400,6 +409,15 @@
         <v>8</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="7"/>
+      <c r="C9" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
test: login with invalid credentials
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/apiTestData.xlsx
+++ b/src/test/resources/testData/apiTestData.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
   <si>
     <t>CT</t>
   </si>
@@ -41,6 +41,12 @@
   </si>
   <si>
     <t>CT008</t>
+  </si>
+  <si>
+    <t>aaaa</t>
+  </si>
+  <si>
+    <t>CT010</t>
   </si>
 </sst>
 </file>
@@ -60,14 +66,15 @@
       <name val="Arial"/>
     </font>
     <font>
+      <b/>
+      <sz val="18.0"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
-      <b/>
-      <sz val="18.0"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -108,10 +115,10 @@
     <xf quotePrefix="1" borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
+    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -120,8 +127,8 @@
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" vertical="bottom"/>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -340,7 +347,7 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="10.0"/>
+    <col customWidth="1" min="1" max="1" width="15.38"/>
     <col customWidth="1" min="2" max="2" width="37.63"/>
     <col customWidth="1" min="3" max="3" width="19.13"/>
   </cols>
@@ -413,9 +420,16 @@
       <c r="A9" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="7"/>
-      <c r="C9" s="1" t="s">
-        <v>8</v>
+      <c r="B9" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
test: delete user account
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/apiTestData.xlsx
+++ b/src/test/resources/testData/apiTestData.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="40">
   <si>
     <t>CT</t>
   </si>
@@ -128,6 +128,9 @@
   </si>
   <si>
     <t>QWQWQ</t>
+  </si>
+  <si>
+    <t>CT012</t>
   </si>
 </sst>
 </file>
@@ -854,9 +857,15 @@
       <c r="Z11" s="3"/>
     </row>
     <row r="12">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
+      <c r="A12" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>30</v>
+      </c>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>

</xml_diff>

<commit_message>
test: add user account tests and improve code consistency
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/apiTestData.xlsx
+++ b/src/test/resources/testData/apiTestData.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="42">
   <si>
     <t>CT</t>
   </si>
@@ -131,6 +131,12 @@
   </si>
   <si>
     <t>CT012</t>
+  </si>
+  <si>
+    <t>CT013</t>
+  </si>
+  <si>
+    <t>CT014</t>
   </si>
 </sst>
 </file>
@@ -891,24 +897,60 @@
       <c r="Z12" s="3"/>
     </row>
     <row r="13">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
-      <c r="J13" s="3"/>
-      <c r="K13" s="3"/>
-      <c r="L13" s="3"/>
-      <c r="M13" s="3"/>
-      <c r="N13" s="3"/>
-      <c r="O13" s="3"/>
-      <c r="P13" s="3"/>
-      <c r="Q13" s="3"/>
-      <c r="R13" s="3"/>
+      <c r="A13" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F13" s="2">
+        <v>14.0</v>
+      </c>
+      <c r="G13" s="2">
+        <v>12.0</v>
+      </c>
+      <c r="H13" s="2">
+        <v>1970.0</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="L13" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="M13" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="N13" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="O13" s="2">
+        <v>12345.0</v>
+      </c>
+      <c r="P13" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q13" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="R13" s="2">
+        <v>1.11111111E8</v>
+      </c>
       <c r="S13" s="3"/>
       <c r="T13" s="3"/>
       <c r="U13" s="3"/>
@@ -919,24 +961,60 @@
       <c r="Z13" s="3"/>
     </row>
     <row r="14">
-      <c r="A14" s="3"/>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
-      <c r="J14" s="3"/>
-      <c r="K14" s="3"/>
-      <c r="L14" s="3"/>
-      <c r="M14" s="3"/>
-      <c r="N14" s="3"/>
-      <c r="O14" s="3"/>
-      <c r="P14" s="3"/>
-      <c r="Q14" s="3"/>
-      <c r="R14" s="3"/>
+      <c r="A14" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F14" s="2">
+        <v>14.0</v>
+      </c>
+      <c r="G14" s="2">
+        <v>12.0</v>
+      </c>
+      <c r="H14" s="2">
+        <v>1970.0</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="L14" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="M14" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="N14" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="O14" s="2">
+        <v>12345.0</v>
+      </c>
+      <c r="P14" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q14" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="R14" s="2">
+        <v>1.11111111E8</v>
+      </c>
       <c r="S14" s="3"/>
       <c r="T14" s="3"/>
       <c r="U14" s="3"/>

</xml_diff>